<commit_message>
Edit line chart and add additional comments
</commit_message>
<xml_diff>
--- a/Test_Data/DimSchedule.xlsx
+++ b/Test_Data/DimSchedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/55cd0139eebd0c53/Desktop/Github Repo/PaupackLaxStatTracking/Test_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{A57E856F-5E94-46A2-BFC7-6C0CCD06CE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00DB7C8B-897F-4851-8F0B-AB9678A0AB93}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{A57E856F-5E94-46A2-BFC7-6C0CCD06CE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50D7F2F3-C6E2-4AC7-A48A-4A50ED5AE888}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-5010" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB70DB8-0B8D-4C6D-8574-C9CE147F1544}"/>
+    <workbookView xWindow="28680" yWindow="-5010" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB70DB8-0B8D-4C6D-8574-C9CE147F1544}"/>
   </bookViews>
   <sheets>
     <sheet name="DimSchedule" sheetId="2" r:id="rId1"/>

</xml_diff>